<commit_message>
Updated language as indicated in the PR. Added additional test cases to neagtive and positive.
</commit_message>
<xml_diff>
--- a/rules/CORE-000236/negative/01/data/unit-test-coreid-CG0079-negative.xlsx
+++ b/rules/CORE-000236/negative/01/data/unit-test-coreid-CG0079-negative.xlsx
@@ -543,7 +543,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F11"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="str">
@@ -685,9 +685,89 @@
         <v>2012-12-17</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="2">
+        <v>4</v>
+      </c>
+      <c r="B8" s="2" t="str">
+        <v>mh.xpt</v>
+      </c>
+      <c r="C8" s="2" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D8" s="2">
+        <v>5</v>
+      </c>
+      <c r="E8" s="2" t="str">
+        <v>MHSTDTC</v>
+      </c>
+      <c r="F8" s="2" t="str">
+        <v>2004-05-28</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2">
+        <v>4</v>
+      </c>
+      <c r="B9" s="2" t="str">
+        <v>dm.xpt</v>
+      </c>
+      <c r="C9" s="2" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D9" s="2">
+        <v>5</v>
+      </c>
+      <c r="E9" s="2" t="str">
+        <v>RFSTDTC</v>
+      </c>
+      <c r="F9" s="2" t="str">
+        <v>2004-05-28</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2">
+        <v>5</v>
+      </c>
+      <c r="B10" s="2" t="str">
+        <v>mh.xpt</v>
+      </c>
+      <c r="C10" s="2" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D10" s="2">
+        <v>9</v>
+      </c>
+      <c r="E10" s="2" t="str">
+        <v>MHSTDTC</v>
+      </c>
+      <c r="F10" s="2" t="str">
+        <v>2006-08-20T10:30</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2">
+        <v>5</v>
+      </c>
+      <c r="B11" s="2" t="str">
+        <v>dm.xpt</v>
+      </c>
+      <c r="C11" s="2" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D11" s="2">
+        <v>9</v>
+      </c>
+      <c r="E11" s="2" t="str">
+        <v>RFSTDTC</v>
+      </c>
+      <c r="F11" s="2" t="str">
+        <v>2006-08-20T10:00</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F11"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1029,8 +1109,8 @@
       <c r="D5" s="4" t="str">
         <v>1115</v>
       </c>
-      <c r="E5" s="4" t="str">
-        <v>2012-11-30</v>
+      <c r="E5" s="7" t="str">
+        <v>2004-05-28</v>
       </c>
       <c r="F5" s="4" t="str">
         <v>2013-01-23</v>
@@ -1109,7 +1189,7 @@
       <c r="D6" s="4" t="str">
         <v>1211</v>
       </c>
-      <c r="E6" s="7" t="str">
+      <c r="E6" s="8" t="str">
         <v>2012-11-15</v>
       </c>
       <c r="F6" s="4" t="str">
@@ -1349,8 +1429,8 @@
       <c r="D9" s="4" t="str">
         <v>1383</v>
       </c>
-      <c r="E9" s="4" t="str">
-        <v>2013-02-04</v>
+      <c r="E9" s="7" t="str">
+        <v>2006-08-20T10:00</v>
       </c>
       <c r="F9" s="4" t="str">
         <v>2013-08-06</v>
@@ -1749,7 +1829,7 @@
       <c r="D14" s="4" t="str">
         <v>1236</v>
       </c>
-      <c r="E14" s="8" t="str">
+      <c r="E14" s="9" t="str">
         <v>2013-09-21</v>
       </c>
       <c r="F14" s="4" t="str">
@@ -2590,7 +2670,7 @@
       <c r="F5" s="4" t="str">
         <v>SYMPTOM ONSET</v>
       </c>
-      <c r="G5" s="4" t="str">
+      <c r="G5" s="7" t="str">
         <v>2004-05-28</v>
       </c>
       <c r="H5" s="4">
@@ -2616,7 +2696,7 @@
       <c r="F6" s="4" t="str">
         <v>SYMPTOM ONSET</v>
       </c>
-      <c r="G6" s="8" t="str">
+      <c r="G6" s="9" t="str">
         <v>2012-11-20</v>
       </c>
       <c r="H6" s="4">
@@ -2694,8 +2774,8 @@
       <c r="F9" s="4" t="str">
         <v>SYMPTOM ONSET</v>
       </c>
-      <c r="G9" s="4" t="str">
-        <v>2006-08-20</v>
+      <c r="G9" s="7" t="str">
+        <v>2006-08-20T10:30</v>
       </c>
       <c r="H9" s="4">
         <v>-2360</v>
@@ -2824,7 +2904,7 @@
       <c r="F14" s="4" t="str">
         <v>SYMPTOM ONSET</v>
       </c>
-      <c r="G14" s="8" t="str">
+      <c r="G14" s="9" t="str">
         <v>2013-09-25</v>
       </c>
       <c r="H14" s="4">
@@ -3006,7 +3086,7 @@
       <c r="F21" s="4" t="str">
         <v>SYMPTOM ONSET</v>
       </c>
-      <c r="G21" s="8" t="str">
+      <c r="G21" s="9" t="str">
         <v>2012-12-20</v>
       </c>
       <c r="H21" s="4">

</xml_diff>